<commit_message>
Documenta os recuos e reversões da Selic nas atas de 2003–2015
Quatro ciclos de corte seguido de volta da taxa, com tabela,
narrativas das atas e gráfico do stop-and-go.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_atas_copom_2001_2026.xlsx
+++ b/output/resumo_atas_copom_2001_2026.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ciclos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anual" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recuos_2003_2015" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anual" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -591,7 +592,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Ajuste e reconstrução de credibilidade</t>
+          <t>Primeiro recuo e reversão (16% → 19,75%)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -643,7 +644,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Afrouxamento e choque internacional</t>
+          <t>Cortes longos e reversão de 2008</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -695,7 +696,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Resposta à crise e retomada</t>
+          <t>Crise: corte a 8,75% e início da volta</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -747,7 +748,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Nova matriz e perda de âncora</t>
+          <t>Nova matriz: recuo a 7,25% e volta forçada</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1057,6 +1058,266 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Episódio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cortes (atas)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Patamar antes</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Piso</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Corte p.p.</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>1ª alta</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pico depois</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Meses até reverter</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Retorno</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1 — desinflação interrompida</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>86ª–95ª</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>26,50</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>16,00</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>100ª (15/09/2004)</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>19,75 (108ª)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>5,1</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>reversão parcial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2 — cortes longos e alta de 2008</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>112ª–129ª</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>19,75</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>8,50</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>134ª (16/04/2008)</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>13,75 (137ª)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>7,4</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>reversão parcial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3 — crise e quase-retorno a 13,75%</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>140ª–144ª</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>8,75</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>5,00</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>150ª (28/04/2010)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>12,50 (160ª)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>9,2</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>quase retornou</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4 — nova matriz e retorno acima do ponto de partida</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>161ª–170ª</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>12,50</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>7,25</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>5,25</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>174ª (17/04/2013)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>14,25 (192ª)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>6,2</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>retornou e superou</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2350,7 +2611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Lista os lapsos contínuos da Selic de 2003 a 2016
Cada intervalo vai até a véspera da reunião que inverte o
sentido, com datas, extensão e taxas de partida e chegada.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_atas_copom_2001_2026.xlsx
+++ b/output/resumo_atas_copom_2001_2026.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ciclos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recuos_2003_2015" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anual" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lapsos_2003_2016" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recuos_2003_2015" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anual" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1063,6 +1064,492 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lapso</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentido</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Início</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fim</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Extensão</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Selic início</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Selic fim</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Δ p.p.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>aumento</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>01/01/2003</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>22/07/2003</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>6 meses e 22 dias</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>26,50</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>+1,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>redução</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>23/07/2003</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2004</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>1 ano, 1 mês e 23 dias</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>26,50</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>16,00</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>−10,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>aumento</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>15/09/2004</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2005</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>11 meses e 30 dias</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>16,00</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>19,75</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>+3,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>redução</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2005</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>15/04/2008</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>2 anos, 7 meses e 2 dias</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>19,75</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>−8,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>aumento</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>16/04/2008</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>20/01/2009</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>9 meses e 5 dias</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>+2,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>redução</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>21/01/2009</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>27/04/2010</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>1 ano, 3 meses e 7 dias</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>8,75</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>−5,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>aumento</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>28/04/2010</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>30/08/2011</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1 ano, 4 meses e 3 dias</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>8,75</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>12,50</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>+3,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>redução</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>31/08/2011</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>16/04/2013</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>1 ano, 7 meses e 17 dias</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>12,50</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>7,25</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>−5,25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>aumento</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>17/04/2013</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>18/10/2016</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>3 anos, 6 meses e 2 dias</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>7,25</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>14,25</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>+7,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>redução</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>19/10/2016</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>31/12/2016</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>2 meses e 13 dias</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>14,25</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>−0,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1317,7 +1804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2611,7 +3098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Publica os 161 patamares da Selic com dias de pregão
Meta do Copom (SGS 432) desde 05/03/1999 e calendário SGS 11:
termo inicial, termo final e número de pregões em cada lapso.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_atas_copom_2001_2026.xlsx
+++ b/output/resumo_atas_copom_2001_2026.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ciclos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lapsos_2003_2016" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recuos_2003_2015" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anual" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lapsos_pregao" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lapsos_2003_2016" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recuos_2003_2015" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anual" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reunioes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1064,6 +1065,4401 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E162"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lapso</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Selic Copom (% a.a.)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Termo inicial</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Termo final</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Dias com pregão</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>05/03/1999</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>24/03/1999</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>42,00</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>25/03/1999</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>05/04/1999</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>39,50</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>06/04/1999</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>14/04/1999</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>34,00</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>15/04/1999</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>28/04/1999</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>32,00</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>29/04/1999</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>07/05/1999</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>10/05/1999</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>12/05/1999</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>27,00</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>13/05/1999</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>19/05/1999</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>23,50</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>20/05/1999</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>08/06/1999</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>22,00</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>09/06/1999</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>23/06/1999</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>21,00</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>24/06/1999</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>28/07/1999</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>19,50</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>29/07/1999</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>22/09/1999</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>23/09/1999</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>28/03/2000</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>18,50</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>29/03/2000</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>20/06/2000</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>17,50</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>21/06/2000</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>07/07/2000</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>17,00</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>10/07/2000</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>19/07/2000</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>16,50</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>20/07/2000</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>20/12/2000</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>15,75</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>21/12/2000</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>17/01/2001</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>15,25</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>18/01/2001</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>21/03/2001</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>15,75</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>22/03/2001</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>18/04/2001</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>16,25</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>19/04/2001</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>23/05/2001</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>16,75</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>24/05/2001</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>20/06/2001</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>18,25</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>21/06/2001</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>18/07/2001</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>19/07/2001</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>20/02/2002</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>18,75</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>21/02/2002</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>20/03/2002</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>18,50</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>21/03/2002</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>17/07/2002</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>18,00</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>18/07/2002</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>14/10/2002</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>21,00</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>15/10/2002</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>20/11/2002</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>22,00</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>21/11/2002</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>18/12/2002</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>19/12/2002</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>22/01/2003</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>25,50</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>23/01/2003</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>19/02/2003</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>26,50</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>20/02/2003</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>18/06/2003</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>26,00</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>20/06/2003</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>23/07/2003</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>24,50</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>24/07/2003</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>20/08/2003</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>22,00</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>21/08/2003</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>17/09/2003</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>18/09/2003</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>22/10/2003</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>23/10/2003</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>19/11/2003</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>17,50</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>20/11/2003</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>17/12/2003</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>16,50</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>18/12/2003</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2004</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>16,25</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>18/03/2004</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>14/04/2004</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>16,00</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>15/04/2004</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>15/09/2004</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>16,25</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>16/09/2004</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2004</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>16,75</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>21/10/2004</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>17/11/2004</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>17,25</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>18/11/2004</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>15/12/2004</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>17,75</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>16/12/2004</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>19/01/2005</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>18,25</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>20/01/2005</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>16/02/2005</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>18,75</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>17/02/2005</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>16/03/2005</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>19,25</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2005</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>20/04/2005</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>19,50</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>22/04/2005</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>18/05/2005</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>19,75</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>19/05/2005</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2005</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>19,50</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>15/09/2005</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>19/10/2005</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2005</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>23/11/2005</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>18,50</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>24/11/2005</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>14/12/2005</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>18,00</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>15/12/2005</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>18/01/2006</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>17,25</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>19/01/2006</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>08/03/2006</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>16,50</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>09/03/2006</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>19/04/2006</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>15,75</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>20/04/2006</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2006</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>15,25</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>01/06/2006</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>19/07/2006</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>14,75</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>20/07/2006</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>30/08/2006</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>14,25</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>31/08/2006</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>18/10/2006</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>19/10/2006</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>29/11/2006</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>13,25</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>30/11/2006</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>24/01/2007</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>13,00</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>25/01/2007</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>07/03/2007</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>12,75</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>08/03/2007</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>18/04/2007</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>12,50</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>19/04/2007</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>06/06/2007</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>08/06/2007</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>18/07/2007</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>11,50</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>19/07/2007</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>05/09/2007</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>06/09/2007</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>16/04/2008</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>11,75</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>17/04/2008</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2008</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>12,25</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>05/06/2008</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>23/07/2008</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>13,00</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>24/07/2008</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>10/09/2008</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>11/09/2008</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>21/01/2009</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>12,75</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>22/01/2009</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>11/03/2009</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>12/03/2009</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>29/04/2009</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>10,25</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>30/04/2009</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>10/06/2009</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>9,25</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>12/06/2009</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>22/07/2009</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>8,75</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>23/07/2009</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>28/04/2010</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>9,50</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>29/04/2010</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>09/06/2010</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>10,25</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>10/06/2010</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>21/07/2010</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>10,75</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>22/07/2010</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>19/01/2011</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>20/01/2011</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>02/03/2011</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>11,75</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>03/03/2011</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>20/04/2011</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>25/04/2011</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>08/06/2011</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>12,25</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>09/06/2011</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>20/07/2011</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>12,50</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>21/07/2011</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>31/08/2011</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>01/09/2011</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>19/10/2011</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>11,50</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>20/10/2011</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>30/11/2011</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>11,00</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>01/12/2011</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>18/01/2012</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>19/01/2012</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>07/03/2012</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>9,75</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>08/03/2012</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>18/04/2012</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>9,00</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>19/04/2012</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>30/05/2012</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>8,50</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>31/05/2012</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>11/07/2012</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>8,00</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>12/07/2012</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>29/08/2012</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>7,50</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>30/08/2012</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>10/10/2012</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>7,25</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>11/10/2012</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>17/04/2013</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>7,50</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>18/04/2013</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>29/05/2013</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>8,00</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2013</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>10/07/2013</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>8,50</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>11/07/2013</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>28/08/2013</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>9,00</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>29/08/2013</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>09/10/2013</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>9,50</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>10/10/2013</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>27/11/2013</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>10,00</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>28/11/2013</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>15/01/2014</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>16/01/2014</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>26/02/2014</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>10,75</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>27/02/2014</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>02/04/2014</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>11,00</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>03/04/2014</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>29/10/2014</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2014</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>03/12/2014</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>11,75</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>04/12/2014</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>21/01/2015</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>12,25</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>22/01/2015</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>04/03/2015</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>12,75</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>05/03/2015</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>29/04/2015</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>13,25</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>30/04/2015</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2015</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>05/06/2015</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>29/07/2015</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>14,25</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>30/07/2015</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>19/10/2016</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>14,00</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2016</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>30/11/2016</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>01/12/2016</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>11/01/2017</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>13,00</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>12/01/2017</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>22/02/2017</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>12,25</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>23/02/2017</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2017</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>13/04/2017</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>31/05/2017</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>10,25</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>01/06/2017</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>26/07/2017</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>9,25</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>27/07/2017</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>06/09/2017</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>8,25</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>08/09/2017</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>25/10/2017</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>7,50</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>26/10/2017</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>06/12/2017</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>7,00</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>07/12/2017</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>07/02/2018</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>6,75</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>08/02/2018</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>21/03/2018</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>6,50</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>22/03/2018</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>31/07/2019</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>341</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>6,00</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>01/08/2019</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>18/09/2019</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>5,50</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>19/09/2019</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2019</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>5,00</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>31/10/2019</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>11/12/2019</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>4,50</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>12/12/2019</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>05/02/2020</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>4,25</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>06/02/2020</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>18/03/2020</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>3,75</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>19/03/2020</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>06/05/2020</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>3,00</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2020</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>17/06/2020</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>2,25</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>18/06/2020</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>05/08/2020</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>2,00</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>06/08/2020</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2021</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>153</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>2,75</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>18/03/2021</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>05/05/2021</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>3,50</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>06/05/2021</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>16/06/2021</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>4,25</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>17/06/2021</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>04/08/2021</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>5,25</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>05/08/2021</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>22/09/2021</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>6,25</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>23/09/2021</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>27/10/2021</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>7,75</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>28/10/2021</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>08/12/2021</t>
+        </is>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>9,25</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>09/12/2021</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>02/02/2022</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>10,75</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>03/02/2022</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>16/03/2022</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>11,75</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2022</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>04/05/2022</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>12,75</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>05/05/2022</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>15/06/2022</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>13,25</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>17/06/2022</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>03/08/2022</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>13,75</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>04/08/2022</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>02/08/2023</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>13,25</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>03/08/2023</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>20/09/2023</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>12,75</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>21/09/2023</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>01/11/2023</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>12,25</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>03/11/2023</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>13/12/2023</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>11,75</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>14/12/2023</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>31/01/2024</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>01/02/2024</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>20/03/2024</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>149</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>10,75</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>21/03/2024</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>08/05/2024</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>09/05/2024</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>18/09/2024</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>10,75</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>19/09/2024</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>06/11/2024</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>11,25</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>07/11/2024</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>11/12/2024</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>153</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>12,25</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>12/12/2024</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>29/01/2025</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>13,25</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>30/01/2025</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>19/03/2025</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>14,25</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>20/03/2025</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2025</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>14,75</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>08/05/2025</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>18/06/2025</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>15,00</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>20/06/2025</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>14,75</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>14,50</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>14,25</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>14,00</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1544,7 +5940,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1804,7 +6200,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3098,7 +7494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>